<commit_message>
Fix the phase-space generator's claims and regenerate the artifacts
The report said it measured rendering cost, but frame timing is limited
by the 120 Hz display. The KPI tiles showed one case beside a 36-run
count, and a linear histogram hid the 191 intervals of 30 ms or more.

- Purpose now says the benchmark tests whether the scene fits the frame
  budget.
- The dashboard note states the worst frame and age p95 across all runs.
- The histogram count axis is log-scaled; zero bins become gaps.
- The template's 68 unused shared strings are dropped; a test fails if
  they return.
- "Cases x repeats" states the recorded run count.
- Template paths are required; the tests read one from an environment
  variable instead of a path on the author's machine.
- The generator accepts run schema v1 and v2.
- Artifacts regenerated from the unchanged 36 runs; summary.json is
  byte-identical in content.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/acceptance/phase-space-v1/artifacts/phase-space-dashboard.xlsx
+++ b/docs/acceptance/phase-space-v1/artifacts/phase-space-dashboard.xlsx
@@ -34,212 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="68">
-  <si>
-    <t>Website Analytics Dashboard</t>
-  </si>
-  <si>
-    <t>SELECTED REPORTING PERIOD</t>
-  </si>
-  <si>
-    <t>DATA CURRENT THROUGH</t>
-  </si>
-  <si>
-    <t>Dashboard</t>
-  </si>
-  <si>
-    <t>ACTIVE USERS</t>
-  </si>
-  <si>
-    <t>NEW USERS</t>
-  </si>
-  <si>
-    <t>30-DAY RETENTION</t>
-  </si>
-  <si>
-    <t>TRIAL-TO-PAID</t>
-  </si>
-  <si>
-    <t>vs prior</t>
-  </si>
-  <si>
-    <t>vs target</t>
-  </si>
-  <si>
-    <t>SESSIONS / USER</t>
-  </si>
-  <si>
-    <t>MONTHLY RECURRING REVENUE</t>
-  </si>
-  <si>
-    <t>BOUNCE RATE</t>
-  </si>
-  <si>
-    <t>MRR / ACTIVE USER</t>
-  </si>
-  <si>
-    <t>ACTIVE USERS — ACTUAL VS TARGET</t>
-  </si>
-  <si>
-    <t>MRR — ACTUAL VS TARGET</t>
-  </si>
-  <si>
-    <t>CONVERSION FUNNEL — SELECTED PERIOD</t>
-  </si>
-  <si>
-    <t>MRR MIX BY SEGMENT</t>
-  </si>
-  <si>
-    <t>SELECTED-PERIOD VARIANCE</t>
-  </si>
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Goal</t>
-  </si>
-  <si>
-    <t>Actual</t>
-  </si>
-  <si>
-    <t>Target</t>
-  </si>
-  <si>
-    <t>Absolute Variance</t>
-  </si>
-  <si>
-    <t>Variance %</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Status is direction-aware: most metrics favor higher results, while Bounce Rate explicitly favors lower results. Watch thresholds are within 5% of target.</t>
-  </si>
-  <si>
-    <t>Synthetic illustrative data for template use.</t>
-  </si>
-  <si>
-    <t>Data &amp; Targets</t>
-  </si>
-  <si>
-    <t>HOW TO USE</t>
-  </si>
-  <si>
-    <t>Paste or replace synthetic monthly actuals and targets in yellow cells B15:P26. Keep dates as real month-start dates.</t>
-  </si>
-  <si>
-    <t>Choose Selected Period in C8. Dashboard KPIs, comparisons, variance status, funnel, and mix recalculate from that period.</t>
-  </si>
-  <si>
-    <t>Selected Period</t>
-  </si>
-  <si>
-    <t>Data Current Through</t>
-  </si>
-  <si>
-    <t>Source Note</t>
-  </si>
-  <si>
-    <t>Synthetic generic example data for template review; replace only yellow inputs.</t>
-  </si>
-  <si>
-    <t>MONTHLY ACTUALS &amp; TARGETS — EDIT YELLOW CELLS</t>
-  </si>
-  <si>
-    <t>Period</t>
-  </si>
-  <si>
-    <t>Active Users</t>
-  </si>
-  <si>
-    <t>New Users</t>
-  </si>
-  <si>
-    <t>30-Day Retention</t>
-  </si>
-  <si>
-    <t>Trial-to-Paid Conversion</t>
-  </si>
-  <si>
-    <t>Sessions / User</t>
-  </si>
-  <si>
-    <t>MRR</t>
-  </si>
-  <si>
-    <t>Bounce Rate</t>
-  </si>
-  <si>
-    <t>Active Users Target</t>
-  </si>
-  <si>
-    <t>New Users Target</t>
-  </si>
-  <si>
-    <t>Retention Target</t>
-  </si>
-  <si>
-    <t>Conversion Target</t>
-  </si>
-  <si>
-    <t>Sessions Target</t>
-  </si>
-  <si>
-    <t>MRR Target</t>
-  </si>
-  <si>
-    <t>Bounce Target</t>
-  </si>
-  <si>
-    <t>FUNNEL DRIVERS — EDIT YELLOW CELLS</t>
-  </si>
-  <si>
-    <t>SEGMENT MIX — EDIT YELLOW CELLS</t>
-  </si>
-  <si>
-    <t>Driver</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Segment</t>
-  </si>
-  <si>
-    <t>Share</t>
-  </si>
-  <si>
-    <t>Visitors per active user</t>
-  </si>
-  <si>
-    <t>Enterprise</t>
-  </si>
-  <si>
-    <t>Visitor to signup</t>
-  </si>
-  <si>
-    <t>Midmarket</t>
-  </si>
-  <si>
-    <t>Signup completion</t>
-  </si>
-  <si>
-    <t>SMB</t>
-  </si>
-  <si>
-    <t>Workspace activation</t>
-  </si>
-  <si>
-    <t>Self-Svc</t>
-  </si>
-  <si>
-    <t>Activation to paid</t>
-  </si>
-  <si>
-    <t>Share Check</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1903,6 +1698,7 @@
       <ns0:valAx>
         <ns0:axId val="2009006557"/>
         <ns0:scaling>
+          <ns0:logBase val="10"/>
           <ns0:orientation val="minMax"/>
         </ns0:scaling>
         <ns0:delete val="0"/>
@@ -2578,7 +2374,7 @@
     <row r="4" spans="2:17" ht="20" customHeight="1" ns3:dyDescent="0.15">
       <c r="B4" s="46" t="inlineStr">
         <is>
-          <t>Build 3745369692fd; 36/36 runs. Dirty runs are non-quotable. See Runs and report for provenance.</t>
+          <t>Build 3745369692fd; 36/36 runs. Tiles show the selected case; worst across all runs: frame p95 10.43 ms, age p95 40.97 ms. Dirty runs are non-quotable.</t>
         </is>
       </c>
       <c r="C4" s="46"/>
@@ -4020,7 +3816,7 @@
       </c>
       <c r="C11" s="84" t="inlineStr">
         <is>
-          <t>Build 3745369692fd; 36/36 runs. Dirty runs are non-quotable. See Runs and report for provenance.</t>
+          <t>Build 3745369692fd; 36/36 runs. Tiles show the selected case; worst across all runs: frame p95 10.43 ms, age p95 40.97 ms. Dirty runs are non-quotable.</t>
         </is>
       </c>
       <c r="D11" s="84"/>

</xml_diff>